<commit_message>
Annotation workbook: optional price, crowding and scenery columns
The focused set measures four aspects. A piece like 'there were no much
crowd when we reach there' is plainly about crowding, and having nowhere to
record that makes the task feel broken even though a blank is the correct
answer for all four columns.

--all-aspects adds the other three. Anything recorded there is a bonus, not
part of the headline measurement -- price, crowding and scenery already score
0.98, 0.90 and 0.91 with the plain word list, which is why the sampling
excluded them. The importer adds any column the gold set lacks rather than
dropping a verdict somebody actually made.

The instructions tab counts the columns it is describing, so the four-aspect
and seven-aspect workbooks no longer both claim to have four.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/travellens/reports/LABEL_THESE_annotator1.xlsx
+++ b/travellens/reports/LABEL_THESE_annotator1.xlsx
@@ -519,7 +519,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>You are reading one PIECE of a review and saying whether the visitor is complaining about any of four things.</t>
+          <t>You are reading one PIECE of a review and saying whether the visitor is complaining about any of 4 things.</t>
         </is>
       </c>
     </row>
@@ -529,35 +529,35 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>The four columns</t>
+          <t>The 4 columns</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Roads &amp; access   roads, parking, buses, the walk, signage, finding it</t>
+          <t>Roads &amp; access     roads, parking, buses, the walk, signage, finding it</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Cleanliness      litter, plastic, smells, upkeep</t>
+          <t>Cleanliness        litter, plastic, smells, upkeep</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Facilities       toilets, food, seating, shelter, bins, guides</t>
+          <t>Facilities         toilets, food, seating, shelter, bins, guides</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Safety           slippery ground, deep water, wildlife, warnings</t>
+          <t>Safety             slippery ground, deep water, wildlife, warnings</t>
         </is>
       </c>
     </row>

</xml_diff>